<commit_message>
Embed cached formula results in HS code summary
LibreOffice recalculation is unavailable in this environment - it also
times out on the pre-existing Czech Healthcare workbook, so the failure is
environmental rather than a problem with this file.

All 18 formula cells were recomputed and asserted in Python, then their
results were written into the sheet XML as cached values. The formulas
themselves are untouched, so Excel still recalculates on open if the
weights or values are edited; the cached results simply make the numbers
visible to previewers and other non-Excel readers.

Verified: allocated net weights sum to 23,00 kg and gross weights to
34,00 kg (delivery note totals), value totals 15 031,00 EUR, quantity
totals 16 pcs, and no cell evaluates to an error.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PHz4DZBZeyTQiJwPU31Y1f
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Hitachi_Energy_139788.xlsx
+++ b/output/HS_Code_Summary_Hitachi_Energy_139788.xlsx
@@ -790,10 +790,12 @@
       </c>
       <c r="D17" s="9">
         <f>$B$13*F17/$F$23</f>
+        <v>2.1299980041248086</v>
         <v/>
       </c>
       <c r="E17" s="9">
         <f>$B$14*F17/$F$23</f>
+        <v>3.148692701749717</v>
         <v/>
       </c>
       <c r="F17" s="10" t="n">
@@ -826,10 +828,12 @@
       </c>
       <c r="D18" s="9">
         <f>$B$13*F18/$F$23</f>
+        <v>9.364646397445279</v>
         <v/>
       </c>
       <c r="E18" s="9">
         <f>$B$14*F18/$F$23</f>
+        <v>13.84339032665824</v>
         <v/>
       </c>
       <c r="F18" s="10" t="n">
@@ -862,10 +866,12 @@
       </c>
       <c r="D19" s="9">
         <f>$B$13*F19/$F$23</f>
+        <v>2.7726698157141905</v>
         <v/>
       </c>
       <c r="E19" s="9">
         <f>$B$14*F19/$F$23</f>
+        <v>4.09872929279489</v>
         <v/>
       </c>
       <c r="F19" s="10" t="n">
@@ -898,10 +904,12 @@
       </c>
       <c r="D20" s="9">
         <f>$B$13*F20/$F$23</f>
+        <v>4.988357394717584</v>
         <v/>
       </c>
       <c r="E20" s="9">
         <f>$B$14*F20/$F$23</f>
+        <v>7.374093540017298</v>
         <v/>
       </c>
       <c r="F20" s="10" t="n">
@@ -934,10 +942,12 @@
       </c>
       <c r="D21" s="9">
         <f>$B$13*F21/$F$23</f>
+        <v>2.455924422859424</v>
         <v/>
       </c>
       <c r="E21" s="9">
         <f>$B$14*F21/$F$23</f>
+        <v>3.6304969729226264</v>
         <v/>
       </c>
       <c r="F21" s="10" t="n">
@@ -970,10 +980,12 @@
       </c>
       <c r="D22" s="9">
         <f>$B$13*F22/$F$23</f>
+        <v>1.2884039651387134</v>
         <v/>
       </c>
       <c r="E22" s="9">
         <f>$B$14*F22/$F$23</f>
+        <v>1.9045971658572285</v>
         <v/>
       </c>
       <c r="F22" s="10" t="n">
@@ -1003,18 +1015,22 @@
       </c>
       <c r="C23" s="13">
         <f>SUM(C17:C22)</f>
+        <v>16.0</v>
         <v/>
       </c>
       <c r="D23" s="14">
         <f>SUM(D17:D22)</f>
+        <v>23.0</v>
         <v/>
       </c>
       <c r="E23" s="14">
         <f>SUM(E17:E22)</f>
+        <v>34.0</v>
         <v/>
       </c>
       <c r="F23" s="15">
         <f>SUM(F17:F22)</f>
+        <v>15031.0</v>
         <v/>
       </c>
       <c r="G23" s="16" t="n"/>
@@ -1398,12 +1414,14 @@
       <c r="C11" s="16" t="n"/>
       <c r="D11" s="24">
         <f>SUM(D4:D10)</f>
+        <v>16.0</v>
         <v/>
       </c>
       <c r="E11" s="16" t="n"/>
       <c r="F11" s="16" t="n"/>
       <c r="G11" s="25">
         <f>SUM(G4:G10)</f>
+        <v>15031.0</v>
         <v/>
       </c>
     </row>

</xml_diff>